<commit_message>
Add slippage modeling + out-of-sample walk-forward + band auto-suggest
Realism/honesty improvements from a deeper review:
- config: new slippage_percent_per_side; cost check now subtracts fees AND
  slippage on both sides (config.yaml + config.amd.yaml updated)
- backtest: fills now slippage-adjusted (buy higher, sell lower), so results
  are conservative not rosy (demo P&L drops $9.25 -> $7.38)
- backtest --suggest-band: recommends a band from price percentiles (stop guessing)
- backtest --walkforward: fits band on early data, tests on later unseen data,
  and flags likely overfit (the #1 way backtests lie)
- compare_windows --csv: run with your own data, no keys needed
- tests: +4 (slippage, suggest_band, walk_forward x2) = 42 total
- workbook + setup guide updated (slippage row, 42 passed)
</commit_message>
<xml_diff>
--- a/docs/Trading_Bot_Setup.xlsx
+++ b/docs/Trading_Bot_Setup.xlsx
@@ -1442,11 +1442,11 @@
         </is>
       </c>
       <c r="E4" s="23" t="n">
-        <v>-3.85</v>
+        <v>-5.77</v>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>-2.14</t>
+          <t>-3.21</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -1473,15 +1473,15 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>1.86</v>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>-0.03</v>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>-0.02</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -1512,11 +1512,11 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>9.25</v>
+        <v>7.38</v>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>5.14</t>
+          <t>4.10</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="E7" s="8" t="n">
-        <v>17.63</v>
+        <v>15.84</v>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>9.80</t>
+          <t>8.80</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -1582,11 +1582,11 @@
         </is>
       </c>
       <c r="E8" s="24" t="n">
-        <v>25.12</v>
+        <v>23.41</v>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>13.95</t>
+          <t>13.00</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -1617,11 +1617,11 @@
         </is>
       </c>
       <c r="E9" s="8" t="n">
-        <v>4.93</v>
+        <v>3.93</v>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -1652,11 +1652,11 @@
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>12.54</v>
+        <v>10</v>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>5.22</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -1687,11 +1687,11 @@
         </is>
       </c>
       <c r="E11" s="8" t="n">
-        <v>16.12</v>
+        <v>12.86</v>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>5.37</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -1722,11 +1722,11 @@
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>19.7</v>
+        <v>15.71</v>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>5.47</t>
+          <t>4.36</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -1781,7 +1781,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last run: 38 passed. CI re-runs these on every push to GitHub.</t>
+          <t>Last run: 42 passed. CI re-runs these on every push to GitHub.</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>$9.25</t>
+          <t>$7.38</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>$15.0</t>
+          <t>$15.04</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>5.14%</t>
+          <t>4.1%</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Run safety tests (expect: 38 passed)</t>
+          <t>Run safety tests (expect: 42 passed)</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -4591,7 +4591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4718,109 +4718,109 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>band_low</t>
+          <t>slippage_percent_per_side</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>90000</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Bottom of your band (buy zone). Set from the backtest.</t>
+          <t>Price you wanted vs got. The main cost for commission-free stocks. Don't set to 0.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>band_high</t>
+          <t>band_low</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>110000</t>
+          <t>90000</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Top of your band (sell zone). Must exceed band_low.</t>
+          <t>Bottom of your band (buy zone). Set from the backtest.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>grid_levels</t>
+          <t>band_high</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>110000</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Rungs to split the band into. More = more, smaller trades.</t>
+          <t>Top of your band (sell zone). Must exceed band_low.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>profit_target_percent</t>
+          <t>grid_levels</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Aim per cycle. Must clear ~0.5% fee. Below ~0.7% is refused.</t>
+          <t>Rungs to split the band into. More = more, smaller trades.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>order_size_usd</t>
+          <t>profit_target_percent</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Dollars per individual buy order.</t>
+          <t>Aim per cycle. Must clear ~0.5% fee. Below ~0.7% is refused.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>max_position_usd</t>
+          <t>order_size_usd</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Largest holdings value allowed. Hard cap.</t>
+          <t>Dollars per individual buy order.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>max_deployed_usd</t>
+          <t>max_position_usd</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -4830,158 +4830,175 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Largest total in open buys + holdings. Hard cap.</t>
+          <t>Largest holdings value allowed. Hard cap.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>max_open_orders</t>
+          <t>max_deployed_usd</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Most resting orders at once.</t>
+          <t>Largest total in open buys + holdings. Hard cap.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="21" t="inlineStr">
         <is>
-          <t>daily_loss_limit_usd</t>
+          <t>max_open_orders</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>If today's loss (realized + unrealized) hits this, halt + cancel.</t>
+          <t>Most resting orders at once.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
         <is>
-          <t>breakout_guard_enabled</t>
+          <t>daily_loss_limit_usd</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Stop new buys if price leaves the band. Leave ON.</t>
+          <t>If today's loss (realized + unrealized) hits this, halt + cancel.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="21" t="inlineStr">
         <is>
-          <t>breakout_flatten</t>
+          <t>breakout_guard_enabled</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>On breakout, also SELL everything to cash. Start false.</t>
+          <t>Stop new buys if price leaves the band. Leave ON.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="21" t="inlineStr">
         <is>
-          <t>loop_interval_seconds</t>
+          <t>breakout_flatten</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Seconds between decisions. 30-60 is plenty.</t>
+          <t>On breakout, also SELL everything to cash. Start false.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="21" t="inlineStr">
         <is>
-          <t>alerts_enabled</t>
+          <t>loop_interval_seconds</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Webhook alert on guard/kill/loss. Needs ALERT_WEBHOOK_URL.</t>
+          <t>Seconds between decisions. 30-60 is plenty.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>log_dir</t>
+          <t>alerts_enabled</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>logs</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Where timestamped logs go.</t>
+          <t>Webhook alert on guard/kill/loss. Needs ALERT_WEBHOOK_URL.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>state_file</t>
+          <t>log_dir</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>state/bot_state.json</t>
+          <t>logs</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Where the bot saves memory between restarts.</t>
+          <t>Where timestamped logs go.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="21" t="inlineStr">
         <is>
+          <t>state_file</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>state/bot_state.json</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Where the bot saves memory between restarts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
           <t>kill_switch_file</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>KILL</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>If this file exists, the bot stops and cancels everything.</t>
         </is>
@@ -5035,7 +5052,7 @@
         <v>100000</v>
       </c>
       <c r="C2" t="n">
-        <v>-5.0136</v>
+        <v>-5.0561</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -5049,7 +5066,7 @@
         <v>106291.43</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.7796999999999999</v>
+        <v>-0.8394</v>
       </c>
       <c r="D3" t="n">
         <v>11.3246</v>
@@ -5063,7 +5080,7 @@
         <v>108089.46</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.2226</v>
+        <v>-0.2977</v>
       </c>
       <c r="D4" t="n">
         <v>14.561</v>
@@ -5077,7 +5094,7 @@
         <v>104729.88</v>
       </c>
       <c r="C5" t="n">
-        <v>-1.4983</v>
+        <v>-1.5878</v>
       </c>
       <c r="D5" t="n">
         <v>8.5138</v>
@@ -5091,7 +5108,7 @@
         <v>99675.75999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>-4.9907</v>
+        <v>-5.0934</v>
       </c>
       <c r="D6" t="n">
         <v>-0.5836</v>
@@ -5105,7 +5122,7 @@
         <v>97106.72</v>
       </c>
       <c r="C7" t="n">
-        <v>-7.4475</v>
+        <v>-7.564</v>
       </c>
       <c r="D7" t="n">
         <v>-5.2079</v>
@@ -5119,7 +5136,7 @@
         <v>98110.84</v>
       </c>
       <c r="C8" t="n">
-        <v>-6.2867</v>
+        <v>-6.4038</v>
       </c>
       <c r="D8" t="n">
         <v>-3.4005</v>
@@ -5133,7 +5150,7 @@
         <v>100080.16</v>
       </c>
       <c r="C9" t="n">
-        <v>-4.4977</v>
+        <v>-4.6309</v>
       </c>
       <c r="D9" t="n">
         <v>0.1443</v>
@@ -5147,7 +5164,7 @@
         <v>99750.13</v>
       </c>
       <c r="C10" t="n">
-        <v>-4.7782</v>
+        <v>-4.9112</v>
       </c>
       <c r="D10" t="n">
         <v>-0.4498</v>
@@ -5161,7 +5178,7 @@
         <v>96784.53</v>
       </c>
       <c r="C11" t="n">
-        <v>-7.6707</v>
+        <v>-7.8172</v>
       </c>
       <c r="D11" t="n">
         <v>-5.7878</v>
@@ -5175,7 +5192,7 @@
         <v>94309.12</v>
       </c>
       <c r="C12" t="n">
-        <v>-10.5322</v>
+        <v>-10.6773</v>
       </c>
       <c r="D12" t="n">
         <v>-10.2436</v>
@@ -5189,7 +5206,7 @@
         <v>95812.48</v>
       </c>
       <c r="C13" t="n">
-        <v>-8.7943</v>
+        <v>-8.940300000000001</v>
       </c>
       <c r="D13" t="n">
         <v>-7.5375</v>
@@ -5203,7 +5220,7 @@
         <v>101429.62</v>
       </c>
       <c r="C14" t="n">
-        <v>-3.2016</v>
+        <v>-3.3656</v>
       </c>
       <c r="D14" t="n">
         <v>2.5733</v>
@@ -5217,7 +5234,7 @@
         <v>107304.58</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1604</v>
+        <v>-0.0355</v>
       </c>
       <c r="D15" t="n">
         <v>13.1482</v>
@@ -5231,7 +5248,7 @@
         <v>108809.09</v>
       </c>
       <c r="C16" t="n">
-        <v>0.5707</v>
+        <v>0.3746</v>
       </c>
       <c r="D16" t="n">
         <v>15.8564</v>
@@ -5245,7 +5262,7 @@
         <v>104673.44</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.9326</v>
+        <v>-1.143</v>
       </c>
       <c r="D17" t="n">
         <v>8.4122</v>
@@ -5259,7 +5276,7 @@
         <v>98152.88</v>
       </c>
       <c r="C18" t="n">
-        <v>-5.6879</v>
+        <v>-5.9109</v>
       </c>
       <c r="D18" t="n">
         <v>-3.3248</v>
@@ -5273,7 +5290,7 @@
         <v>94123.24000000001</v>
       </c>
       <c r="C19" t="n">
-        <v>-10.2993</v>
+        <v>-10.535</v>
       </c>
       <c r="D19" t="n">
         <v>-10.5782</v>
@@ -5287,7 +5304,7 @@
         <v>94831.34</v>
       </c>
       <c r="C20" t="n">
-        <v>-9.2155</v>
+        <v>-9.4666</v>
       </c>
       <c r="D20" t="n">
         <v>-9.303599999999999</v>
@@ -5301,7 +5318,7 @@
         <v>98253.03999999999</v>
       </c>
       <c r="C21" t="n">
-        <v>-5.3761</v>
+        <v>-5.6443</v>
       </c>
       <c r="D21" t="n">
         <v>-3.1445</v>
@@ -5315,7 +5332,7 @@
         <v>100474.3</v>
       </c>
       <c r="C22" t="n">
-        <v>-3.4165</v>
+        <v>-3.7009</v>
       </c>
       <c r="D22" t="n">
         <v>0.8537</v>
@@ -5329,7 +5346,7 @@
         <v>99661.98</v>
       </c>
       <c r="C23" t="n">
-        <v>-4.1069</v>
+        <v>-4.3909</v>
       </c>
       <c r="D23" t="n">
         <v>-0.6084000000000001</v>
@@ -5343,7 +5360,7 @@
         <v>97732.57000000001</v>
       </c>
       <c r="C24" t="n">
-        <v>-5.8285</v>
+        <v>-6.1266</v>
       </c>
       <c r="D24" t="n">
         <v>-4.0814</v>
@@ -5357,7 +5374,7 @@
         <v>98141.56</v>
       </c>
       <c r="C25" t="n">
-        <v>-5.3557</v>
+        <v>-5.6541</v>
       </c>
       <c r="D25" t="n">
         <v>-3.3452</v>
@@ -5371,7 +5388,7 @@
         <v>102041.04</v>
       </c>
       <c r="C26" t="n">
-        <v>-1.9358</v>
+        <v>-2.251</v>
       </c>
       <c r="D26" t="n">
         <v>3.6739</v>
@@ -5385,7 +5402,7 @@
         <v>106673.81</v>
       </c>
       <c r="C27" t="n">
-        <v>0.7761</v>
+        <v>0.4443</v>
       </c>
       <c r="D27" t="n">
         <v>12.0129</v>
@@ -5399,7 +5416,7 @@
         <v>107710.99</v>
       </c>
       <c r="C28" t="n">
-        <v>1.0175</v>
+        <v>0.6705</v>
       </c>
       <c r="D28" t="n">
         <v>13.8798</v>
@@ -5413,7 +5430,7 @@
         <v>103381.81</v>
       </c>
       <c r="C29" t="n">
-        <v>-0.9042</v>
+        <v>-1.2652</v>
       </c>
       <c r="D29" t="n">
         <v>6.0872</v>
@@ -5427,7 +5444,7 @@
         <v>96427.7</v>
       </c>
       <c r="C30" t="n">
-        <v>-6.8892</v>
+        <v>-7.2772</v>
       </c>
       <c r="D30" t="n">
         <v>-6.4301</v>
@@ -5441,7 +5458,7 @@
         <v>91917.57000000001</v>
       </c>
       <c r="C31" t="n">
-        <v>-12.7674</v>
+        <v>-13.1675</v>
       </c>
       <c r="D31" t="n">
         <v>-14.5484</v>
@@ -5455,7 +5472,7 @@
         <v>92884.03999999999</v>
       </c>
       <c r="C32" t="n">
-        <v>-11.3417</v>
+        <v>-11.7425</v>
       </c>
       <c r="D32" t="n">
         <v>-12.8087</v>
@@ -5469,7 +5486,7 @@
         <v>97820.57000000001</v>
       </c>
       <c r="C33" t="n">
-        <v>-5.1298</v>
+        <v>-5.5488</v>
       </c>
       <c r="D33" t="n">
         <v>-3.923</v>
@@ -5483,7 +5500,7 @@
         <v>102318.06</v>
       </c>
       <c r="C34" t="n">
-        <v>-1.1033</v>
+        <v>-1.5395</v>
       </c>
       <c r="D34" t="n">
         <v>4.1725</v>
@@ -5497,7 +5514,7 @@
         <v>103203.88</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.5553</v>
+        <v>-1.0069</v>
       </c>
       <c r="D35" t="n">
         <v>5.767</v>
@@ -5511,7 +5528,7 @@
         <v>101228.47</v>
       </c>
       <c r="C36" t="n">
-        <v>-1.8801</v>
+        <v>-2.346</v>
       </c>
       <c r="D36" t="n">
         <v>2.2112</v>
@@ -5525,7 +5542,7 @@
         <v>99828.14</v>
       </c>
       <c r="C37" t="n">
-        <v>-3.0702</v>
+        <v>-3.5355</v>
       </c>
       <c r="D37" t="n">
         <v>-0.3093</v>
@@ -5539,7 +5556,7 @@
         <v>101321.49</v>
       </c>
       <c r="C38" t="n">
-        <v>-1.801</v>
+        <v>-2.267</v>
       </c>
       <c r="D38" t="n">
         <v>2.3787</v>
@@ -5553,7 +5570,7 @@
         <v>104363.8</v>
       </c>
       <c r="C39" t="n">
-        <v>0.2385</v>
+        <v>-0.2436</v>
       </c>
       <c r="D39" t="n">
         <v>7.8548</v>
@@ -5567,7 +5584,7 @@
         <v>105213.18</v>
       </c>
       <c r="C40" t="n">
-        <v>0.7106</v>
+        <v>0.2282</v>
       </c>
       <c r="D40" t="n">
         <v>9.383699999999999</v>
@@ -5581,7 +5598,7 @@
         <v>101597.34</v>
       </c>
       <c r="C41" t="n">
-        <v>-1.4173</v>
+        <v>-1.9136</v>
       </c>
       <c r="D41" t="n">
         <v>2.8752</v>
@@ -5595,7 +5612,7 @@
         <v>95369.74000000001</v>
       </c>
       <c r="C42" t="n">
-        <v>-7.5151</v>
+        <v>-8.023400000000001</v>
       </c>
       <c r="D42" t="n">
         <v>-8.3345</v>
@@ -5609,7 +5626,7 @@
         <v>91245.14999999999</v>
       </c>
       <c r="C43" t="n">
-        <v>-13.1623</v>
+        <v>-13.6827</v>
       </c>
       <c r="D43" t="n">
         <v>-15.7587</v>
@@ -5623,7 +5640,7 @@
         <v>92666.46000000001</v>
       </c>
       <c r="C44" t="n">
-        <v>-11.0657</v>
+        <v>-11.5871</v>
       </c>
       <c r="D44" t="n">
         <v>-13.2004</v>
@@ -5637,7 +5654,7 @@
         <v>98655.94</v>
       </c>
       <c r="C45" t="n">
-        <v>-3.5671</v>
+        <v>-4.1074</v>
       </c>
       <c r="D45" t="n">
         <v>-2.4193</v>
@@ -5651,7 +5668,7 @@
         <v>104632.28</v>
       </c>
       <c r="C46" t="n">
-        <v>0.8355</v>
+        <v>0.2627</v>
       </c>
       <c r="D46" t="n">
         <v>8.338100000000001</v>
@@ -5665,7 +5682,7 @@
         <v>106445.85</v>
       </c>
       <c r="C47" t="n">
-        <v>1.8434</v>
+        <v>1.27</v>
       </c>
       <c r="D47" t="n">
         <v>11.6025</v>
@@ -5679,7 +5696,7 @@
         <v>103863.64</v>
       </c>
       <c r="C48" t="n">
-        <v>0.4083</v>
+        <v>-0.1643</v>
       </c>
       <c r="D48" t="n">
         <v>6.9546</v>
@@ -5693,7 +5710,7 @@
         <v>100308.76</v>
       </c>
       <c r="C49" t="n">
-        <v>-2.0647</v>
+        <v>-2.6511</v>
       </c>
       <c r="D49" t="n">
         <v>0.5558</v>
@@ -5707,7 +5724,7 @@
         <v>99261.12</v>
       </c>
       <c r="C50" t="n">
-        <v>-2.9551</v>
+        <v>-3.541</v>
       </c>
       <c r="D50" t="n">
         <v>-1.33</v>
@@ -5721,7 +5738,7 @@
         <v>100885.28</v>
       </c>
       <c r="C51" t="n">
-        <v>-1.5748</v>
+        <v>-2.1614</v>
       </c>
       <c r="D51" t="n">
         <v>1.5935</v>
@@ -5735,7 +5752,7 @@
         <v>102142.44</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.5063</v>
+        <v>-1.0935</v>
       </c>
       <c r="D52" t="n">
         <v>3.8564</v>
@@ -5749,7 +5766,7 @@
         <v>100191.93</v>
       </c>
       <c r="C53" t="n">
-        <v>-2.164</v>
+        <v>-2.7503</v>
       </c>
       <c r="D53" t="n">
         <v>0.3455</v>
@@ -5763,7 +5780,7 @@
         <v>95651.47</v>
       </c>
       <c r="C54" t="n">
-        <v>-6.7417</v>
+        <v>-7.3407</v>
       </c>
       <c r="D54" t="n">
         <v>-7.8274</v>
@@ -5777,7 +5794,7 @@
         <v>92405.82000000001</v>
       </c>
       <c r="C55" t="n">
-        <v>-11.0024</v>
+        <v>-11.6143</v>
       </c>
       <c r="D55" t="n">
         <v>-13.6695</v>
@@ -5791,7 +5808,7 @@
         <v>94018.89</v>
       </c>
       <c r="C56" t="n">
-        <v>-8.6229</v>
+        <v>-9.236000000000001</v>
       </c>
       <c r="D56" t="n">
         <v>-10.766</v>
@@ -5805,7 +5822,7 @@
         <v>100158.29</v>
       </c>
       <c r="C57" t="n">
-        <v>-1.8941</v>
+        <v>-2.5408</v>
       </c>
       <c r="D57" t="n">
         <v>0.2849</v>
@@ -5819,7 +5836,7 @@
         <v>106524.41</v>
       </c>
       <c r="C58" t="n">
-        <v>2.3348</v>
+        <v>1.6708</v>
       </c>
       <c r="D58" t="n">
         <v>11.7439</v>
@@ -5833,7 +5850,7 @@
         <v>108477.59</v>
       </c>
       <c r="C59" t="n">
-        <v>2.8683</v>
+        <v>2.1889</v>
       </c>
       <c r="D59" t="n">
         <v>15.2597</v>
@@ -5847,7 +5864,7 @@
         <v>105032.12</v>
       </c>
       <c r="C60" t="n">
-        <v>1.6547</v>
+        <v>0.9609</v>
       </c>
       <c r="D60" t="n">
         <v>9.0578</v>
@@ -5861,7 +5878,7 @@
         <v>99519.37</v>
       </c>
       <c r="C61" t="n">
-        <v>-2.1386</v>
+        <v>-2.8455</v>
       </c>
       <c r="D61" t="n">
         <v>-0.8651</v>
@@ -5875,7 +5892,7 @@
         <v>96372.67</v>
       </c>
       <c r="C62" t="n">
-        <v>-5.311</v>
+        <v>-6.0313</v>
       </c>
       <c r="D62" t="n">
         <v>-6.5292</v>
@@ -5889,7 +5906,7 @@
         <v>97134.97</v>
       </c>
       <c r="C63" t="n">
-        <v>-4.4298</v>
+        <v>-5.1505</v>
       </c>
       <c r="D63" t="n">
         <v>-5.1571</v>
@@ -5903,7 +5920,7 @@
         <v>99448.38</v>
       </c>
       <c r="C64" t="n">
-        <v>-2.0497</v>
+        <v>-2.7867</v>
       </c>
       <c r="D64" t="n">
         <v>-0.9929</v>
@@ -5917,7 +5934,7 @@
         <v>99847.14</v>
       </c>
       <c r="C65" t="n">
-        <v>-1.7108</v>
+        <v>-2.448</v>
       </c>
       <c r="D65" t="n">
         <v>-0.2751</v>
@@ -5931,7 +5948,7 @@
         <v>97494.73</v>
       </c>
       <c r="C66" t="n">
-        <v>-3.8647</v>
+        <v>-4.6158</v>
       </c>
       <c r="D66" t="n">
         <v>-4.5095</v>
@@ -5945,7 +5962,7 @@
         <v>95135.12</v>
       </c>
       <c r="C67" t="n">
-        <v>-6.5924</v>
+        <v>-7.3421</v>
       </c>
       <c r="D67" t="n">
         <v>-8.7568</v>
@@ -5959,7 +5976,7 @@
         <v>96294.73</v>
       </c>
       <c r="C68" t="n">
-        <v>-5.2519</v>
+        <v>-6.0023</v>
       </c>
       <c r="D68" t="n">
         <v>-6.6695</v>
@@ -5973,7 +5990,7 @@
         <v>101481.68</v>
       </c>
       <c r="C69" t="n">
-        <v>-0.1724</v>
+        <v>-0.9405</v>
       </c>
       <c r="D69" t="n">
         <v>2.667</v>
@@ -5987,7 +6004,7 @@
         <v>107175.3</v>
       </c>
       <c r="C70" t="n">
-        <v>3.1101</v>
+        <v>2.3101</v>
       </c>
       <c r="D70" t="n">
         <v>12.9155</v>
@@ -6001,7 +6018,7 @@
         <v>108746.94</v>
       </c>
       <c r="C71" t="n">
-        <v>3.5388</v>
+        <v>2.7385</v>
       </c>
       <c r="D71" t="n">
         <v>15.7445</v>
@@ -6015,7 +6032,7 @@
         <v>104647.31</v>
       </c>
       <c r="C72" t="n">
-        <v>2.0378</v>
+        <v>1.2233</v>
       </c>
       <c r="D72" t="n">
         <v>8.3652</v>
@@ -6029,7 +6046,7 @@
         <v>97911.21000000001</v>
       </c>
       <c r="C73" t="n">
-        <v>-2.9355</v>
+        <v>-3.7775</v>
       </c>
       <c r="D73" t="n">
         <v>-3.7598</v>
@@ -6043,7 +6060,7 @@
         <v>93525.16</v>
       </c>
       <c r="C74" t="n">
-        <v>-8.157299999999999</v>
+        <v>-9.0116</v>
       </c>
       <c r="D74" t="n">
         <v>-11.6547</v>
@@ -6057,7 +6074,7 @@
         <v>94102.17999999999</v>
       </c>
       <c r="C75" t="n">
-        <v>-7.3061</v>
+        <v>-8.1609</v>
       </c>
       <c r="D75" t="n">
         <v>-10.6161</v>
@@ -6071,7 +6088,7 @@
         <v>97879.52</v>
       </c>
       <c r="C76" t="n">
-        <v>-2.8229</v>
+        <v>-3.6951</v>
       </c>
       <c r="D76" t="n">
         <v>-3.8169</v>
@@ -6085,7 +6102,7 @@
         <v>100804.48</v>
       </c>
       <c r="C77" t="n">
-        <v>-0.1509</v>
+        <v>-1.0396</v>
       </c>
       <c r="D77" t="n">
         <v>1.4481</v>
@@ -6099,7 +6116,7 @@
         <v>100573.5</v>
       </c>
       <c r="C78" t="n">
-        <v>-0.3472</v>
+        <v>-1.2358</v>
       </c>
       <c r="D78" t="n">
         <v>1.0323</v>
@@ -6113,7 +6130,7 @@
         <v>98687.92999999999</v>
       </c>
       <c r="C79" t="n">
-        <v>-1.9497</v>
+        <v>-2.8375</v>
       </c>
       <c r="D79" t="n">
         <v>-2.3617</v>
@@ -6127,7 +6144,7 @@
         <v>98597.09</v>
       </c>
       <c r="C80" t="n">
-        <v>-2.0269</v>
+        <v>-2.9146</v>
       </c>
       <c r="D80" t="n">
         <v>-2.5252</v>
@@ -6141,7 +6158,7 @@
         <v>101850.28</v>
       </c>
       <c r="C81" t="n">
-        <v>0.7379</v>
+        <v>-0.1512</v>
       </c>
       <c r="D81" t="n">
         <v>3.3305</v>
@@ -6155,7 +6172,7 @@
         <v>106135.04</v>
       </c>
       <c r="C82" t="n">
-        <v>3.3124</v>
+        <v>2.4068</v>
       </c>
       <c r="D82" t="n">
         <v>11.0431</v>
@@ -6169,7 +6186,7 @@
         <v>107243.01</v>
       </c>
       <c r="C83" t="n">
-        <v>3.7256</v>
+        <v>2.8047</v>
       </c>
       <c r="D83" t="n">
         <v>13.0374</v>
@@ -6183,7 +6200,7 @@
         <v>103152.35</v>
       </c>
       <c r="C84" t="n">
-        <v>1.804</v>
+        <v>0.8691</v>
       </c>
       <c r="D84" t="n">
         <v>5.6742</v>
@@ -6197,7 +6214,7 @@
         <v>96282.44</v>
       </c>
       <c r="C85" t="n">
-        <v>-4.2213</v>
+        <v>-5.1832</v>
       </c>
       <c r="D85" t="n">
         <v>-6.6916</v>
@@ -6211,7 +6228,7 @@
         <v>91649.16</v>
       </c>
       <c r="C86" t="n">
-        <v>-10.3276</v>
+        <v>-11.3014</v>
       </c>
       <c r="D86" t="n">
         <v>-15.0315</v>
@@ -6225,7 +6242,7 @@
         <v>92543.21000000001</v>
       </c>
       <c r="C87" t="n">
-        <v>-9.008800000000001</v>
+        <v>-9.9833</v>
       </c>
       <c r="D87" t="n">
         <v>-13.4222</v>
@@ -6239,7 +6256,7 @@
         <v>97733.83</v>
       </c>
       <c r="C88" t="n">
-        <v>-2.3943</v>
+        <v>-3.3872</v>
       </c>
       <c r="D88" t="n">
         <v>-4.0791</v>
@@ -6253,7 +6270,7 @@
         <v>102773.55</v>
       </c>
       <c r="C89" t="n">
-        <v>2.1195</v>
+        <v>1.1092</v>
       </c>
       <c r="D89" t="n">
         <v>4.9924</v>
@@ -6267,7 +6284,7 @@
         <v>104108.08</v>
       </c>
       <c r="C90" t="n">
-        <v>2.7829</v>
+        <v>1.7571</v>
       </c>
       <c r="D90" t="n">
         <v>7.3945</v>
@@ -6281,7 +6298,7 @@
         <v>102085.73</v>
       </c>
       <c r="C91" t="n">
-        <v>1.659</v>
+        <v>0.6337</v>
       </c>
       <c r="D91" t="n">
         <v>3.7543</v>
@@ -6295,7 +6312,7 @@
         <v>100098.19</v>
       </c>
       <c r="C92" t="n">
-        <v>-0.0049</v>
+        <v>-1.0443</v>
       </c>
       <c r="D92" t="n">
         <v>0.1767</v>
@@ -6309,7 +6326,7 @@
         <v>100848.72</v>
       </c>
       <c r="C93" t="n">
-        <v>0.6329</v>
+        <v>-0.4068</v>
       </c>
       <c r="D93" t="n">
         <v>1.5277</v>
@@ -6323,7 +6340,7 @@
         <v>103493.79</v>
       </c>
       <c r="C94" t="n">
-        <v>2.5908</v>
+        <v>1.5349</v>
       </c>
       <c r="D94" t="n">
         <v>6.2888</v>
@@ -6337,7 +6354,7 @@
         <v>104494.76</v>
       </c>
       <c r="C95" t="n">
-        <v>3.1471</v>
+        <v>2.0909</v>
       </c>
       <c r="D95" t="n">
         <v>8.0906</v>
@@ -6351,7 +6368,7 @@
         <v>101346.24</v>
       </c>
       <c r="C96" t="n">
-        <v>1.205</v>
+        <v>0.1348</v>
       </c>
       <c r="D96" t="n">
         <v>2.4232</v>
@@ -6365,7 +6382,7 @@
         <v>95484.83</v>
       </c>
       <c r="C97" t="n">
-        <v>-4.5464</v>
+        <v>-5.6286</v>
       </c>
       <c r="D97" t="n">
         <v>-8.1273</v>
@@ -6379,7 +6396,7 @@
         <v>91415.8</v>
       </c>
       <c r="C98" t="n">
-        <v>-10.0748</v>
+        <v>-11.1693</v>
       </c>
       <c r="D98" t="n">
         <v>-15.4516</v>
@@ -6393,7 +6410,7 @@
         <v>92735.98</v>
       </c>
       <c r="C99" t="n">
-        <v>-8.1274</v>
+        <v>-9.222899999999999</v>
       </c>
       <c r="D99" t="n">
         <v>-13.0752</v>
@@ -6407,7 +6424,7 @@
         <v>98770.14</v>
       </c>
       <c r="C100" t="n">
-        <v>-0.5993000000000001</v>
+        <v>-1.7137</v>
       </c>
       <c r="D100" t="n">
         <v>-2.2138</v>
@@ -6421,7 +6438,7 @@
         <v>105030.74</v>
       </c>
       <c r="C101" t="n">
-        <v>3.8927</v>
+        <v>2.7458</v>
       </c>
       <c r="D101" t="n">
         <v>9.055300000000001</v>
@@ -6435,7 +6452,7 @@
         <v>107119.01</v>
       </c>
       <c r="C102" t="n">
-        <v>4.8858</v>
+        <v>3.7232</v>
       </c>
       <c r="D102" t="n">
         <v>12.8142</v>
@@ -6449,7 +6466,7 @@
         <v>104442.07</v>
       </c>
       <c r="C103" t="n">
-        <v>3.7148</v>
+        <v>2.5378</v>
       </c>
       <c r="D103" t="n">
         <v>7.9957</v>
@@ -6463,7 +6480,7 @@
         <v>100329.89</v>
       </c>
       <c r="C104" t="n">
-        <v>0.9382</v>
+        <v>-0.2523</v>
       </c>
       <c r="D104" t="n">
         <v>0.5938</v>
@@ -6477,7 +6494,7 @@
         <v>98584.78</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.5449000000000001</v>
+        <v>-1.7347</v>
       </c>
       <c r="D105" t="n">
         <v>-2.5474</v>
@@ -6491,7 +6508,7 @@
         <v>99867.21000000001</v>
       </c>
       <c r="C106" t="n">
-        <v>0.545</v>
+        <v>-0.6453</v>
       </c>
       <c r="D106" t="n">
         <v>-0.239</v>
@@ -6505,7 +6522,7 @@
         <v>101386.15</v>
       </c>
       <c r="C107" t="n">
-        <v>1.8359</v>
+        <v>0.6449</v>
       </c>
       <c r="D107" t="n">
         <v>2.4951</v>
@@ -6519,7 +6536,7 @@
         <v>100087.8</v>
       </c>
       <c r="C108" t="n">
-        <v>0.7325</v>
+        <v>-0.458</v>
       </c>
       <c r="D108" t="n">
         <v>0.158</v>
@@ -6533,7 +6550,7 @@
         <v>96108.81</v>
       </c>
       <c r="C109" t="n">
-        <v>-3.228</v>
+        <v>-4.4315</v>
       </c>
       <c r="D109" t="n">
         <v>-7.0041</v>
@@ -6547,7 +6564,7 @@
         <v>93001.48</v>
       </c>
       <c r="C110" t="n">
-        <v>-7.1388</v>
+        <v>-8.3553</v>
       </c>
       <c r="D110" t="n">
         <v>-12.5973</v>
@@ -6561,7 +6578,7 @@
         <v>94399.53999999999</v>
       </c>
       <c r="C111" t="n">
-        <v>-5.0764</v>
+        <v>-6.294</v>
       </c>
       <c r="D111" t="n">
         <v>-10.0808</v>
@@ -6575,7 +6592,7 @@
         <v>100310.41</v>
       </c>
       <c r="C112" t="n">
-        <v>1.2202</v>
+        <v>-0.0308</v>
       </c>
       <c r="D112" t="n">
         <v>0.5587</v>
@@ -6589,7 +6606,7 @@
         <v>106674.12</v>
       </c>
       <c r="C113" t="n">
-        <v>5.403</v>
+        <v>4.1348</v>
       </c>
       <c r="D113" t="n">
         <v>12.0134</v>
@@ -6603,7 +6620,7 @@
         <v>108753.34</v>
       </c>
       <c r="C114" t="n">
-        <v>5.9285</v>
+        <v>4.6449</v>
       </c>
       <c r="D114" t="n">
         <v>15.756</v>
@@ -6617,7 +6634,7 @@
         <v>105253.49</v>
       </c>
       <c r="C115" t="n">
-        <v>4.7627</v>
+        <v>3.4647</v>
       </c>
       <c r="D115" t="n">
         <v>9.456300000000001</v>
@@ -6631,7 +6648,7 @@
         <v>99343.69</v>
       </c>
       <c r="C116" t="n">
-        <v>0.6971000000000001</v>
+        <v>-0.6139</v>
       </c>
       <c r="D116" t="n">
         <v>-1.1814</v>
@@ -6645,7 +6662,7 @@
         <v>95666.78999999999</v>
       </c>
       <c r="C117" t="n">
-        <v>-3.142</v>
+        <v>-4.4661</v>
       </c>
       <c r="D117" t="n">
         <v>-7.7998</v>
@@ -6659,7 +6676,7 @@
         <v>96200.47</v>
       </c>
       <c r="C118" t="n">
-        <v>-2.5251</v>
+        <v>-3.8494</v>
       </c>
       <c r="D118" t="n">
         <v>-6.8392</v>
@@ -6673,7 +6690,7 @@
         <v>98852.13</v>
       </c>
       <c r="C119" t="n">
-        <v>0.5402</v>
+        <v>-0.7857</v>
       </c>
       <c r="D119" t="n">
         <v>-2.0662</v>
@@ -6687,7 +6704,7 @@
         <v>99981.64999999999</v>
       </c>
       <c r="C120" t="n">
-        <v>1.3885</v>
+        <v>0.0471</v>
       </c>
       <c r="D120" t="n">
         <v>-0.033</v>
@@ -6701,7 +6718,7 @@
         <v>98258.09</v>
       </c>
       <c r="C121" t="n">
-        <v>-0.07630000000000001</v>
+        <v>-1.417</v>
       </c>
       <c r="D121" t="n">
         <v>-3.1354</v>
@@ -6715,7 +6732,7 @@
         <v>96020.36</v>
       </c>
       <c r="C122" t="n">
-        <v>-2.584</v>
+        <v>-3.9385</v>
       </c>
       <c r="D122" t="n">
         <v>-7.1634</v>
@@ -6729,7 +6746,7 @@
         <v>96805.33</v>
       </c>
       <c r="C123" t="n">
-        <v>-1.6766</v>
+        <v>-3.0315</v>
       </c>
       <c r="D123" t="n">
         <v>-5.7504</v>
@@ -6743,7 +6760,7 @@
         <v>101496.03</v>
       </c>
       <c r="C124" t="n">
-        <v>2.8248</v>
+        <v>1.4525</v>
       </c>
       <c r="D124" t="n">
         <v>2.6929</v>
@@ -6757,7 +6774,7 @@
         <v>106945.33</v>
       </c>
       <c r="C125" t="n">
-        <v>6.1507</v>
+        <v>4.7616</v>
       </c>
       <c r="D125" t="n">
         <v>12.5016</v>
@@ -6771,7 +6788,7 @@
         <v>108570.11</v>
       </c>
       <c r="C126" t="n">
-        <v>6.4755</v>
+        <v>5.0711</v>
       </c>
       <c r="D126" t="n">
         <v>15.4262</v>
@@ -6785,7 +6802,7 @@
         <v>104555.56</v>
       </c>
       <c r="C127" t="n">
-        <v>4.9718</v>
+        <v>3.5532</v>
       </c>
       <c r="D127" t="n">
         <v>8.199999999999999</v>
@@ -6799,7 +6816,7 @@
         <v>97684.52</v>
       </c>
       <c r="C128" t="n">
-        <v>-0.2125</v>
+        <v>-1.6586</v>
       </c>
       <c r="D128" t="n">
         <v>-4.1679</v>
@@ -6813,7 +6830,7 @@
         <v>93002.45</v>
       </c>
       <c r="C129" t="n">
-        <v>-5.9433</v>
+        <v>-7.4015</v>
       </c>
       <c r="D129" t="n">
         <v>-12.5956</v>
@@ -6827,7 +6844,7 @@
         <v>93458.12</v>
       </c>
       <c r="C130" t="n">
-        <v>-5.2711</v>
+        <v>-6.7297</v>
       </c>
       <c r="D130" t="n">
         <v>-11.7754</v>
@@ -6841,7 +6858,7 @@
         <v>97561.55</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.2054</v>
+        <v>-1.6816</v>
       </c>
       <c r="D131" t="n">
         <v>-4.3892</v>
@@ -6855,7 +6872,7 @@
         <v>101156.91</v>
       </c>
       <c r="C132" t="n">
-        <v>3.1336</v>
+        <v>1.6406</v>
       </c>
       <c r="D132" t="n">
         <v>2.0824</v>
@@ -6869,7 +6886,7 @@
         <v>101493.48</v>
       </c>
       <c r="C133" t="n">
-        <v>3.4196</v>
+        <v>1.9265</v>
       </c>
       <c r="D133" t="n">
         <v>2.6883</v>
@@ -6883,7 +6900,7 @@
         <v>99648.74000000001</v>
       </c>
       <c r="C134" t="n">
-        <v>1.8519</v>
+        <v>0.3595</v>
       </c>
       <c r="D134" t="n">
         <v>-0.6323</v>
@@ -6897,7 +6914,7 @@
         <v>99040.69</v>
       </c>
       <c r="C135" t="n">
-        <v>1.3351</v>
+        <v>-0.157</v>
       </c>
       <c r="D135" t="n">
         <v>-1.7268</v>
@@ -6911,7 +6928,7 @@
         <v>101607.48</v>
       </c>
       <c r="C136" t="n">
-        <v>3.5165</v>
+        <v>2.0233</v>
       </c>
       <c r="D136" t="n">
         <v>2.8935</v>
@@ -6925,7 +6942,7 @@
         <v>105505.86</v>
       </c>
       <c r="C137" t="n">
-        <v>5.9477</v>
+        <v>4.4382</v>
       </c>
       <c r="D137" t="n">
         <v>9.910500000000001</v>
@@ -6939,7 +6956,7 @@
         <v>106686.32</v>
       </c>
       <c r="C138" t="n">
-        <v>6.6038</v>
+        <v>5.0939</v>
       </c>
       <c r="D138" t="n">
         <v>12.0354</v>
@@ -6953,7 +6970,7 @@
         <v>102890.72</v>
       </c>
       <c r="C139" t="n">
-        <v>4.4944</v>
+        <v>2.9855</v>
       </c>
       <c r="D139" t="n">
         <v>5.2033</v>
@@ -6967,7 +6984,7 @@
         <v>96188.10000000001</v>
       </c>
       <c r="C140" t="n">
-        <v>-1.4946</v>
+        <v>-3.0305</v>
       </c>
       <c r="D140" t="n">
         <v>-6.8614</v>
@@ -6981,7 +6998,7 @@
         <v>91488.83</v>
       </c>
       <c r="C141" t="n">
-        <v>-7.7284</v>
+        <v>-9.2761</v>
       </c>
       <c r="D141" t="n">
         <v>-15.3201</v>
@@ -6995,7 +7012,7 @@
         <v>92306.84</v>
       </c>
       <c r="C142" t="n">
-        <v>-6.5217</v>
+        <v>-8.07</v>
       </c>
       <c r="D142" t="n">
         <v>-13.8477</v>
@@ -7009,7 +7026,7 @@
         <v>97696.98</v>
       </c>
       <c r="C143" t="n">
-        <v>0.3989</v>
+        <v>-1.168</v>
       </c>
       <c r="D143" t="n">
         <v>-4.1454</v>
@@ -7023,7 +7040,7 @@
         <v>103216.42</v>
       </c>
       <c r="C144" t="n">
-        <v>5.1231</v>
+        <v>3.5236</v>
       </c>
       <c r="D144" t="n">
         <v>5.7896</v>
@@ -7037,7 +7054,7 @@
         <v>104967.05</v>
       </c>
       <c r="C145" t="n">
-        <v>6.096</v>
+        <v>4.496</v>
       </c>
       <c r="D145" t="n">
         <v>8.9407</v>
@@ -7051,7 +7068,7 @@
         <v>102898.37</v>
       </c>
       <c r="C146" t="n">
-        <v>4.9464</v>
+        <v>3.3469</v>
       </c>
       <c r="D146" t="n">
         <v>5.2171</v>
@@ -7065,7 +7082,7 @@
         <v>100332.05</v>
       </c>
       <c r="C147" t="n">
-        <v>3.0296</v>
+        <v>1.4161</v>
       </c>
       <c r="D147" t="n">
         <v>0.5977</v>
@@ -7079,7 +7096,7 @@
         <v>100334.38</v>
       </c>
       <c r="C148" t="n">
-        <v>3.0316</v>
+        <v>1.4181</v>
       </c>
       <c r="D148" t="n">
         <v>0.6019</v>
@@ -7093,7 +7110,7 @@
         <v>102570.24</v>
       </c>
       <c r="C149" t="n">
-        <v>4.9317</v>
+        <v>3.3173</v>
       </c>
       <c r="D149" t="n">
         <v>4.6264</v>
@@ -7107,7 +7124,7 @@
         <v>103732.79</v>
       </c>
       <c r="C150" t="n">
-        <v>5.5593</v>
+        <v>3.9295</v>
       </c>
       <c r="D150" t="n">
         <v>6.719</v>
@@ -7121,7 +7138,7 @@
         <v>101100.41</v>
       </c>
       <c r="C151" t="n">
-        <v>3.8318</v>
+        <v>2.1878</v>
       </c>
       <c r="D151" t="n">
         <v>1.9807</v>
@@ -7135,7 +7152,7 @@
         <v>95673.25999999999</v>
       </c>
       <c r="C152" t="n">
-        <v>-1.4928</v>
+        <v>-3.1491</v>
       </c>
       <c r="D152" t="n">
         <v>-7.7881</v>
@@ -7149,7 +7166,7 @@
         <v>91701.21000000001</v>
       </c>
       <c r="C153" t="n">
-        <v>-6.8181</v>
+        <v>-8.486800000000001</v>
       </c>
       <c r="D153" t="n">
         <v>-14.9378</v>
@@ -7163,7 +7180,7 @@
         <v>92900.7</v>
       </c>
       <c r="C154" t="n">
-        <v>-5.0487</v>
+        <v>-6.7182</v>
       </c>
       <c r="D154" t="n">
         <v>-12.7787</v>
@@ -7177,7 +7194,7 @@
         <v>98907.57000000001</v>
       </c>
       <c r="C155" t="n">
-        <v>2.3953</v>
+        <v>0.7069</v>
       </c>
       <c r="D155" t="n">
         <v>-1.9664</v>
@@ -7191,7 +7208,7 @@
         <v>105374.59</v>
       </c>
       <c r="C156" t="n">
-        <v>6.9195</v>
+        <v>5.1985</v>
       </c>
       <c r="D156" t="n">
         <v>9.674300000000001</v>
@@ -7205,7 +7222,7 @@
         <v>107700.69</v>
       </c>
       <c r="C157" t="n">
-        <v>7.8802</v>
+        <v>6.1436</v>
       </c>
       <c r="D157" t="n">
         <v>13.8613</v>
@@ -7219,7 +7236,7 @@
         <v>104944.27</v>
       </c>
       <c r="C158" t="n">
-        <v>6.8296</v>
+        <v>5.0786</v>
       </c>
       <c r="D158" t="n">
         <v>8.899699999999999</v>
@@ -7233,7 +7250,7 @@
         <v>100314.55</v>
       </c>
       <c r="C159" t="n">
-        <v>3.761</v>
+        <v>1.9964</v>
       </c>
       <c r="D159" t="n">
         <v>0.5662</v>
@@ -7247,7 +7264,7 @@
         <v>97900.72</v>
       </c>
       <c r="C160" t="n">
-        <v>1.6791</v>
+        <v>-0.0993</v>
       </c>
       <c r="D160" t="n">
         <v>-3.7787</v>
@@ -7261,7 +7278,7 @@
         <v>98849.00999999999</v>
       </c>
       <c r="C161" t="n">
-        <v>2.7753</v>
+        <v>0.9963</v>
       </c>
       <c r="D161" t="n">
         <v>-2.0718</v>
@@ -7275,7 +7292,7 @@
         <v>100635.58</v>
       </c>
       <c r="C162" t="n">
-        <v>4.183</v>
+        <v>2.3882</v>
       </c>
       <c r="D162" t="n">
         <v>1.144</v>
@@ -7289,7 +7306,7 @@
         <v>100015.21</v>
       </c>
       <c r="C163" t="n">
-        <v>3.6558</v>
+        <v>1.8612</v>
       </c>
       <c r="D163" t="n">
         <v>0.0274</v>
@@ -7303,7 +7320,7 @@
         <v>96637.75</v>
       </c>
       <c r="C164" t="n">
-        <v>0.3684</v>
+        <v>-1.4396</v>
       </c>
       <c r="D164" t="n">
         <v>-6.0521</v>
@@ -7317,7 +7334,7 @@
         <v>93689.3</v>
       </c>
       <c r="C165" t="n">
-        <v>-3.1391</v>
+        <v>-4.9603</v>
       </c>
       <c r="D165" t="n">
         <v>-11.3593</v>
@@ -7331,7 +7348,7 @@
         <v>94842.64999999999</v>
       </c>
       <c r="C166" t="n">
-        <v>-1.4378</v>
+        <v>-3.2598</v>
       </c>
       <c r="D166" t="n">
         <v>-9.283200000000001</v>
@@ -7345,7 +7362,7 @@
         <v>100450.3</v>
       </c>
       <c r="C167" t="n">
-        <v>4.3241</v>
+        <v>2.4689</v>
       </c>
       <c r="D167" t="n">
         <v>0.8105</v>
@@ -7359,7 +7376,7 @@
         <v>106735.79</v>
       </c>
       <c r="C168" t="n">
-        <v>8.4223</v>
+        <v>6.5499</v>
       </c>
       <c r="D168" t="n">
         <v>12.1244</v>

</xml_diff>

<commit_message>
Add multi-symbol screener: rank tickers by out-of-sample result
- screen_symbols.py: for each symbol, auto-fit a band and run the walk-forward
  out-of-sample test, then RANK by honest out-of-sample strategy return.
  Auto-detects crypto (BTC/USD) vs stock (AMD); supports --days/--csv/--simulate.
- tests/test_screen.py: ranking, asset-class inference, graceful data errors (45 total)
- workbook architecture/commands + setup guide updated (45 passed)
</commit_message>
<xml_diff>
--- a/docs/Trading_Bot_Setup.xlsx
+++ b/docs/Trading_Bot_Setup.xlsx
@@ -1781,7 +1781,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Last run: 42 passed. CI re-runs these on every push to GitHub.</t>
+          <t>Last run: 45 passed. CI re-runs these on every push to GitHub.</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2474,19 +2474,43 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Replays the exact strategy over historical/synthetic/CSV data.</t>
+          <t>Replays the strategy; also --suggest-band and --walkforward (out-of-sample).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="21" t="inlineStr">
         <is>
+          <t>compare_windows.py</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Compares strategy vs buy &amp; hold across 30/60/90-day windows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>screen_symbols.py</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Ranks many tickers by honest out-of-sample result; shows what's worth trading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
           <t>tests/</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Automated proof the dangerous parts are correct (38 tests).</t>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Automated proof the dangerous parts are correct (45 tests).</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4188,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Run safety tests (expect: 42 passed)</t>
+          <t>Run safety tests (expect: 45 passed)</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Add start.py: one friendly menu-driven front door (Apple-style simplicity)
- start.py: a single, beautiful launcher. Interactive numbered menu plus
  direct subcommands (health/backtest/dryrun/screen/keys/explain/etc).
  Plain-language framed output, terminal colours with graceful no-TTY
  fallback, emoji-aware box alignment. Auto-detects whether keys are set
  and runs real-data vs demo accordingly. Wraps the existing tools.
- README + SETUP_GUIDE: feature 'python start.py' as the easy button.
- workbook: start.py added to Architecture + a #0 EASY BUTTON command row.
</commit_message>
<xml_diff>
--- a/docs/Trading_Bot_Setup.xlsx
+++ b/docs/Trading_Bot_Setup.xlsx
@@ -2301,7 +2301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2337,178 +2337,190 @@
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>config.yaml</t>
+          <t>start.py</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Your settings. The only file you normally edit.</t>
+          <t>⭐ The easy front door: a friendly menu that runs everything for you.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>bot/config.py</t>
+          <t>config.yaml</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Loads + validates settings. Refuses to run if anything is unsafe.</t>
+          <t>Your settings. The only file you normally edit.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>bot/fees.py</t>
+          <t>bot/config.py</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>The money math: fees, breakeven, net profit after fees.</t>
+          <t>Loads + validates settings. Refuses to run if anything is unsafe.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>bot/grid.py</t>
+          <t>bot/fees.py</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Turns your band into a ladder of buy/sell price rungs.</t>
+          <t>The money math: fees, breakeven, net profit after fees.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>bot/guards.py</t>
+          <t>bot/grid.py</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>The brakes: breakout, daily-loss halt, risk limits, kill switch.</t>
+          <t>Turns your band into a ladder of buy/sell price rungs.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>bot/broker.py</t>
+          <t>bot/guards.py</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Talks to Alpaca (retries, idempotent IDs) + a local simulator for dry-run.</t>
+          <t>The brakes: breakout, daily-loss halt, risk limits, kill switch.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>bot/state.py</t>
+          <t>bot/broker.py</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Saves/reloads the bot's memory; reconciles with Alpaca on restart.</t>
+          <t>Talks to Alpaca (retries, idempotent IDs) + a local simulator for dry-run.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>bot/engine.py</t>
+          <t>bot/state.py</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>The main loop: read price, detect fills, run guards, place orders, log.</t>
+          <t>Saves/reloads the bot's memory; reconciles with Alpaca on restart.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>bot/alerts.py</t>
+          <t>bot/engine.py</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Optional webhook notifications (Discord/Slack/phone).</t>
+          <t>The main loop: read price, detect fills, run guards, place orders, log.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>bot/logging_setup.py</t>
+          <t>bot/alerts.py</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Timestamped, human-readable logs.</t>
+          <t>Optional webhook notifications (Discord/Slack/phone).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>run_bot.py</t>
+          <t>bot/logging_setup.py</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>What you launch. Picks simulator vs Alpaca based on mode.</t>
+          <t>Timestamped, human-readable logs.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>backtest.py</t>
+          <t>run_bot.py</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Replays the strategy; also --suggest-band and --walkforward (out-of-sample).</t>
+          <t>What you launch. Picks simulator vs Alpaca based on mode.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>compare_windows.py</t>
+          <t>backtest.py</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Compares strategy vs buy &amp; hold across 30/60/90-day windows.</t>
+          <t>Replays the strategy; also --suggest-band and --walkforward (out-of-sample).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="21" t="inlineStr">
         <is>
-          <t>screen_symbols.py</t>
+          <t>compare_windows.py</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Ranks many tickers by honest out-of-sample result; shows what's worth trading.</t>
+          <t>Compares strategy vs buy &amp; hold across 30/60/90-day windows.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
         <is>
+          <t>screen_symbols.py</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Ranks many tickers by honest out-of-sample result; shows what's worth trading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
           <t>tests/</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Automated proof the dangerous parts are correct (45 tests).</t>
         </is>
@@ -4124,7 +4136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4166,151 +4178,168 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Install packages</t>
+          <t>⭐ EASY BUTTON: friendly menu (does it all)</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>pip install -r requirements.txt</t>
+          <t>python start.py</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Run safety tests (expect: 45 passed)</t>
+          <t>Install packages</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>python -m pytest -q</t>
+          <t>pip install -r requirements.txt</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Offline backtest (synthetic data)</t>
+          <t>Run safety tests (expect: 45 passed)</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>python backtest.py --simulate</t>
+          <t>python -m pytest -q</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Offline backtest (synthetic data)</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>python backtest.py --simulate</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Dry run, 30 loops (no keys, nothing sent)</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>python run_bot.py --ticks 30</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Create your secrets file</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>cp .env.example .env</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Backtest on REAL last 30 days (needs paper keys)</t>
+          <t>Create your secrets file</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>python backtest.py --days 30</t>
+          <t>cp .env.example .env</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Backtest on REAL last 30 days (needs paper keys)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>python backtest.py --days 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Start PAPER trading (set mode: paper first)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>python run_bot.py</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>STOP immediately (kill switch)</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>touch KILL   (Win: type nul &gt; KILL)</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Re-arm after a kill</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>rm KILL   (Win: del KILL)</t>
         </is>

</xml_diff>